<commit_message>
Actualizar datos de ingresos
</commit_message>
<xml_diff>
--- a/data/reporte_ingresos.xlsx
+++ b/data/reporte_ingresos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Johan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Johan\monitor-ingresos\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4343" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4730" uniqueCount="845">
   <si>
     <t>ID PDV</t>
   </si>
@@ -2289,6 +2289,276 @@
   </si>
   <si>
     <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1090436828_DBD_INGRESO_PDV_35217_23_09_2026_09_00_21.jpg</t>
+  </si>
+  <si>
+    <t>7824689</t>
+  </si>
+  <si>
+    <t>4.891917916666667</t>
+  </si>
+  <si>
+    <t>-74.03327221666667</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:03:00</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1075688960_DBD_INGRESO_PDV_10772_23_09_2026_09_02_59.jpg</t>
+  </si>
+  <si>
+    <t>7824690</t>
+  </si>
+  <si>
+    <t>10.948503333333333</t>
+  </si>
+  <si>
+    <t>-74.78309666666668</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:03:04</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/72098375_DBD_INGRESO_PDV_2638_23_09_2026_09_03_02.jpg</t>
+  </si>
+  <si>
+    <t>7824692</t>
+  </si>
+  <si>
+    <t>4.678341666666666</t>
+  </si>
+  <si>
+    <t>-74.11810999999999</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:03:51</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/80115103_DBD_INGRESO_PDV_22870_23_09_2026_09_03_50.jpg</t>
+  </si>
+  <si>
+    <t>7824694</t>
+  </si>
+  <si>
+    <t>11.225459999999998</t>
+  </si>
+  <si>
+    <t>-74.174025</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:05:22</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1110533250_DBD_INGRESO_PDV_23897_23_09_2026_09_05_21.jpg</t>
+  </si>
+  <si>
+    <t>7824700</t>
+  </si>
+  <si>
+    <t>10.383586666666668</t>
+  </si>
+  <si>
+    <t>-75.46936166666666</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:08:44</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1002247264_DBD_INGRESO_PDV_8379_23_09_2026_09_08_43.jpg</t>
+  </si>
+  <si>
+    <t>7824703</t>
+  </si>
+  <si>
+    <t>4.6848443</t>
+  </si>
+  <si>
+    <t>-74.0790118</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:11:16</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1028865500_DBD_INGRESO_PDV_59330_23_09_2026_09_11_16.jpg</t>
+  </si>
+  <si>
+    <t>7824709</t>
+  </si>
+  <si>
+    <t>7.1154159</t>
+  </si>
+  <si>
+    <t>-73.1202411</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:17:30</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1102716954_DBD_INGRESO_PDV_80680_23_09_2026_09_17_30.jpg</t>
+  </si>
+  <si>
+    <t>7824721</t>
+  </si>
+  <si>
+    <t>4.588721666666667</t>
+  </si>
+  <si>
+    <t>-74.20568666666667</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:27:10</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1014305216_DBD_INGRESO_PDV_79821_23_09_2026_09_27_10.jpg</t>
+  </si>
+  <si>
+    <t>7824731</t>
+  </si>
+  <si>
+    <t>6.1776837</t>
+  </si>
+  <si>
+    <t>-75.5911041</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:32:15</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/71780913_DBD_INGRESO_PDV_30515_23_09_2026_09_32_06.jpg</t>
+  </si>
+  <si>
+    <t>7824732</t>
+  </si>
+  <si>
+    <t>3.3698833594098687</t>
+  </si>
+  <si>
+    <t>-76.5263925679028</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:33:27</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1114813506_DBD_INGRESO_PDV_81696_23_09_2026_09_33_26.jpg</t>
+  </si>
+  <si>
+    <t>7824740</t>
+  </si>
+  <si>
+    <t>3.4726799999999995</t>
+  </si>
+  <si>
+    <t>-76.52827</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:38:15</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/94412336_DBD_INGRESO_PDV_48560_23_09_2026_09_38_15.jpg</t>
+  </si>
+  <si>
+    <t>7824743</t>
+  </si>
+  <si>
+    <t>6.24955507</t>
+  </si>
+  <si>
+    <t>-75.58426619</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:39:53</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1007634699_DBD_INGRESO_PDV_22864_23_09_2026_09_39_51.jpg</t>
+  </si>
+  <si>
+    <t>7824768</t>
+  </si>
+  <si>
+    <t>10.493436666666666</t>
+  </si>
+  <si>
+    <t>-73.26734</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:52:03</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1065626573_DBD_INGRESO_PDV_85091_23_09_2026_09_52_01.jpg</t>
+  </si>
+  <si>
+    <t>7824775</t>
+  </si>
+  <si>
+    <t>4.700948</t>
+  </si>
+  <si>
+    <t>-74.2307263</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:57:30</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1070464010_DBD_INGRESO_PDV_71439_23_09_2026_09_57_29.jpg</t>
+  </si>
+  <si>
+    <t>7824780</t>
+  </si>
+  <si>
+    <t>11.015293333333334</t>
+  </si>
+  <si>
+    <t>-74.82933166666666</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:58:48</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/72257237_DBD_INGRESO_PDV_46344_23_09_2026_09_58_47.jpg</t>
+  </si>
+  <si>
+    <t>7824781</t>
+  </si>
+  <si>
+    <t>4.618398333333333</t>
+  </si>
+  <si>
+    <t>-74.08616833333333</t>
+  </si>
+  <si>
+    <t>23/09/2026 09:59:26</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1233490257_DBD_INGRESO_PDV_5747_23_09_2026_09_59_24.jpg</t>
+  </si>
+  <si>
+    <t>7824926</t>
+  </si>
+  <si>
+    <t>4.7303521</t>
+  </si>
+  <si>
+    <t>-74.0329322</t>
+  </si>
+  <si>
+    <t>23/09/2026 11:04:10</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/11225449_DBD_INGRESO_PDV_71086_23_09_2026_11_04_09.jpg</t>
+  </si>
+  <si>
+    <t>7824935</t>
+  </si>
+  <si>
+    <t>6.250681666666666</t>
+  </si>
+  <si>
+    <t>-75.583835</t>
+  </si>
+  <si>
+    <t>23/09/2026 11:06:42</t>
+  </si>
+  <si>
+    <t>https://dbdplus.accionplus.com/dbdPlus2/webMod/Public/imagenesDBD/4714/77/1035227940_DBD_INGRESO_PDV_81723_23_09_2026_11_06_40.jpg</t>
   </si>
 </sst>
 </file>
@@ -12996,7 +13266,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG43"/>
+  <dimension ref="A1:AG61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
@@ -15971,7 +16241,7 @@
       </c>
       <c r="AG36" s="2"/>
     </row>
-    <row r="37" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>719</v>
       </c>
@@ -15993,10 +16263,6 @@
       <c r="G37" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-      <c r="J37" s="3"/>
-      <c r="K37" s="3"/>
       <c r="L37" s="3" t="s">
         <v>123</v>
       </c>
@@ -16027,16 +16293,9 @@
       <c r="U37" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="V37" s="3"/>
-      <c r="W37" s="3"/>
-      <c r="X37" s="3"/>
-      <c r="Y37" s="3"/>
       <c r="Z37" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="AA37" s="3"/>
-      <c r="AB37" s="3"/>
-      <c r="AC37" s="3"/>
       <c r="AD37" s="3" t="s">
         <v>723</v>
       </c>
@@ -16046,16 +16305,14 @@
       <c r="AF37" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AG37" s="3"/>
-    </row>
-    <row r="38" spans="1:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>724</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="C38" s="3"/>
       <c r="D38" s="3" t="s">
         <v>208</v>
       </c>
@@ -16068,11 +16325,6 @@
       <c r="G38" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-      <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="3"/>
       <c r="M38" s="3" t="s">
         <v>34</v>
       </c>
@@ -16100,16 +16352,9 @@
       <c r="U38" s="3" t="s">
         <v>728</v>
       </c>
-      <c r="V38" s="3"/>
-      <c r="W38" s="3"/>
-      <c r="X38" s="3"/>
-      <c r="Y38" s="3"/>
       <c r="Z38" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="AA38" s="3"/>
-      <c r="AB38" s="3"/>
-      <c r="AC38" s="3"/>
       <c r="AD38" s="3" t="s">
         <v>729</v>
       </c>
@@ -16123,7 +16368,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>730</v>
       </c>
@@ -16145,10 +16390,6 @@
       <c r="G39" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
-      <c r="K39" s="3"/>
       <c r="L39" s="3" t="s">
         <v>123</v>
       </c>
@@ -16179,16 +16420,9 @@
       <c r="U39" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="V39" s="3"/>
-      <c r="W39" s="3"/>
-      <c r="X39" s="3"/>
-      <c r="Y39" s="3"/>
       <c r="Z39" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="AA39" s="3"/>
-      <c r="AB39" s="3"/>
-      <c r="AC39" s="3"/>
       <c r="AD39" s="3" t="s">
         <v>734</v>
       </c>
@@ -16202,7 +16436,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>735</v>
       </c>
@@ -16224,10 +16458,6 @@
       <c r="G40" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H40" s="3"/>
-      <c r="I40" s="3"/>
-      <c r="J40" s="3"/>
-      <c r="K40" s="3"/>
       <c r="L40" s="3" t="s">
         <v>123</v>
       </c>
@@ -16258,16 +16488,9 @@
       <c r="U40" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="V40" s="3"/>
-      <c r="W40" s="3"/>
-      <c r="X40" s="3"/>
-      <c r="Y40" s="3"/>
       <c r="Z40" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="AA40" s="3"/>
-      <c r="AB40" s="3"/>
-      <c r="AC40" s="3"/>
       <c r="AD40" s="3" t="s">
         <v>739</v>
       </c>
@@ -16277,9 +16500,8 @@
       <c r="AF40" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AG40" s="3"/>
-    </row>
-    <row r="41" spans="1:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>740</v>
       </c>
@@ -16301,10 +16523,6 @@
       <c r="G41" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
-      <c r="K41" s="3"/>
       <c r="L41" s="3" t="s">
         <v>123</v>
       </c>
@@ -16335,16 +16553,9 @@
       <c r="U41" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="V41" s="3"/>
-      <c r="W41" s="3"/>
-      <c r="X41" s="3"/>
-      <c r="Y41" s="3"/>
       <c r="Z41" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="AA41" s="3"/>
-      <c r="AB41" s="3"/>
-      <c r="AC41" s="3"/>
       <c r="AD41" s="3" t="s">
         <v>744</v>
       </c>
@@ -16358,7 +16569,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="42" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>745</v>
       </c>
@@ -16380,10 +16591,6 @@
       <c r="G42" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
       <c r="L42" s="3" t="s">
         <v>123</v>
       </c>
@@ -16414,16 +16621,9 @@
       <c r="U42" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="V42" s="3"/>
-      <c r="W42" s="3"/>
-      <c r="X42" s="3"/>
-      <c r="Y42" s="3"/>
       <c r="Z42" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="AA42" s="3"/>
-      <c r="AB42" s="3"/>
-      <c r="AC42" s="3"/>
       <c r="AD42" s="3" t="s">
         <v>749</v>
       </c>
@@ -16437,7 +16637,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="43" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>750</v>
       </c>
@@ -16459,10 +16659,6 @@
       <c r="G43" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="H43" s="3"/>
-      <c r="I43" s="3"/>
-      <c r="J43" s="3"/>
-      <c r="K43" s="3"/>
       <c r="L43" s="3" t="s">
         <v>123</v>
       </c>
@@ -16493,16 +16689,9 @@
       <c r="U43" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="V43" s="3"/>
-      <c r="W43" s="3"/>
-      <c r="X43" s="3"/>
-      <c r="Y43" s="3"/>
       <c r="Z43" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="AA43" s="3"/>
-      <c r="AB43" s="3"/>
-      <c r="AC43" s="3"/>
       <c r="AD43" s="3" t="s">
         <v>754</v>
       </c>
@@ -16512,7 +16701,1203 @@
       <c r="AF43" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AG43" s="3"/>
+    </row>
+    <row r="44" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>755</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M44" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="N44" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="P44" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q44" s="3" t="s">
+        <v>756</v>
+      </c>
+      <c r="R44" s="3" t="s">
+        <v>757</v>
+      </c>
+      <c r="S44" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T44" s="3" t="s">
+        <v>758</v>
+      </c>
+      <c r="U44" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z44" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD44" s="3" t="s">
+        <v>759</v>
+      </c>
+      <c r="AE44" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF44" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG44" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="45" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L45" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M45" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="N45" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="O45" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="P45" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q45" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="R45" s="3" t="s">
+        <v>762</v>
+      </c>
+      <c r="S45" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T45" s="3" t="s">
+        <v>763</v>
+      </c>
+      <c r="U45" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z45" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD45" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="AE45" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF45" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG45" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="46" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L46" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M46" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N46" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="O46" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="P46" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q46" s="3" t="s">
+        <v>766</v>
+      </c>
+      <c r="R46" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="S46" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T46" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="U46" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z46" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD46" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="AE46" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF46" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>770</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>679</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M47" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="N47" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="O47" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="P47" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q47" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="R47" s="3" t="s">
+        <v>772</v>
+      </c>
+      <c r="S47" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T47" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="U47" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z47" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD47" s="3" t="s">
+        <v>774</v>
+      </c>
+      <c r="AE47" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF47" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG47" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="48" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L48" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M48" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="N48" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="O48" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="P48" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q48" s="3" t="s">
+        <v>776</v>
+      </c>
+      <c r="R48" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="S48" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T48" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="U48" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z48" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD48" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="AE48" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF48" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG48" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="49" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L49" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M49" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N49" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O49" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="P49" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q49" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="R49" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="S49" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T49" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="U49" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z49" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD49" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="AE49" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF49" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L50" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M50" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="N50" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="O50" s="3" t="s">
+        <v>350</v>
+      </c>
+      <c r="P50" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q50" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="R50" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="S50" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T50" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="U50" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z50" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD50" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="AE50" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF50" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG50" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="51" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L51" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M51" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="N51" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="O51" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="P51" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q51" s="3" t="s">
+        <v>791</v>
+      </c>
+      <c r="R51" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="S51" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T51" s="3" t="s">
+        <v>793</v>
+      </c>
+      <c r="U51" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z51" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD51" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="AE51" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF51" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG51" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="52" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L52" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M52" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="N52" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="O52" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="P52" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q52" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="R52" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="S52" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T52" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="U52" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z52" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD52" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="AE52" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF52" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG52" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="53" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
+        <v>800</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M53" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="N53" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="O53" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="P53" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q53" s="3" t="s">
+        <v>801</v>
+      </c>
+      <c r="R53" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="S53" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T53" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="U53" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z53" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD53" s="3" t="s">
+        <v>804</v>
+      </c>
+      <c r="AE53" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF53" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="54" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L54" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M54" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="N54" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="O54" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="P54" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q54" s="3" t="s">
+        <v>806</v>
+      </c>
+      <c r="R54" s="3" t="s">
+        <v>807</v>
+      </c>
+      <c r="S54" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T54" s="3" t="s">
+        <v>808</v>
+      </c>
+      <c r="U54" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z54" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD54" s="3" t="s">
+        <v>809</v>
+      </c>
+      <c r="AE54" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF54" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="55" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>810</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L55" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M55" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="N55" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="O55" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="P55" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q55" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="R55" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="S55" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T55" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="U55" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z55" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD55" s="3" t="s">
+        <v>814</v>
+      </c>
+      <c r="AE55" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF55" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="56" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L56" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M56" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="N56" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="O56" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="P56" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q56" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="R56" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="S56" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T56" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="U56" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z56" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD56" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="AE56" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF56" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="57" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>820</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L57" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="N57" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="O57" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="P57" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q57" s="3" t="s">
+        <v>821</v>
+      </c>
+      <c r="R57" s="3" t="s">
+        <v>822</v>
+      </c>
+      <c r="S57" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T57" s="3" t="s">
+        <v>823</v>
+      </c>
+      <c r="U57" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z57" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD57" s="3" t="s">
+        <v>824</v>
+      </c>
+      <c r="AE57" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF57" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>825</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L58" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M58" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="N58" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="O58" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="P58" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q58" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="R58" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="S58" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T58" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="U58" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z58" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD58" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="AE58" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF58" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG58" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="59" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>830</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L59" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M59" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N59" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="O59" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="P59" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q59" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="R59" s="3" t="s">
+        <v>832</v>
+      </c>
+      <c r="S59" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T59" s="3" t="s">
+        <v>833</v>
+      </c>
+      <c r="U59" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z59" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD59" s="3" t="s">
+        <v>834</v>
+      </c>
+      <c r="AE59" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF59" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG59" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="60" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>835</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L60" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M60" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N60" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="O60" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="P60" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q60" s="3" t="s">
+        <v>836</v>
+      </c>
+      <c r="R60" s="3" t="s">
+        <v>837</v>
+      </c>
+      <c r="S60" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T60" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="U60" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z60" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD60" s="3" t="s">
+        <v>839</v>
+      </c>
+      <c r="AE60" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF60" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG60" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="61" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>840</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L61" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="M61" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="N61" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="O61" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="P61" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q61" s="3" t="s">
+        <v>841</v>
+      </c>
+      <c r="R61" s="3" t="s">
+        <v>842</v>
+      </c>
+      <c r="S61" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="T61" s="3" t="s">
+        <v>843</v>
+      </c>
+      <c r="U61" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="Z61" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="AD61" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="AE61" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF61" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG61" s="3" t="s">
+        <v>68</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AG36"/>

</xml_diff>